<commit_message>
Web: actualizar landing con iPhone rico + secciones científicas
- iPhone flotante rediseñado: anillo SVG (88% kcal), barras de macros,
  lista de comidas del día, coach IA adaptado al tipo de sesión,
  racha e hidratación
- Nueva sección "17 estudios. 0 pseudociencia." con 4 science claim cards
- Stats bar con datos científicos (82% Mifflin-St Jeor, 8 sesiones...)
- Nueva sección "Por qué elegirla" con 4 diferenciadores vs competencia
- Copy hero y sección IA actualizados con brand voice científica
- 2 FAQ nuevas sobre metodología y periodización deportiva
- Footer: link a /guides/metodologia.html
- Tildes corregidas en 6 textos del HTML

Incluye también cambios previos en stash: finanzas, marketing carousels,
brand voice guide, content-source, instagram-commenter.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finances/Cals2Gains_Finances.xlsx
+++ b/finances/Cals2Gains_Finances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Judit\Documents\Cals2Gains\finances\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DC4DF75-7CFE-494A-B7BA-5AAA0E0C60A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477A0307-AAB0-4B8F-B495-35AD85C11C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="4110" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gastos" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="128">
   <si>
     <t>Fecha</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Seq: 1-13389522137</t>
   </si>
   <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
     <t>Mes</t>
   </si>
   <si>
@@ -246,9 +243,6 @@
     <t>Anual</t>
   </si>
   <si>
-    <t>Pendiente pago</t>
-  </si>
-  <si>
     <t>Expo (EAS)</t>
   </si>
   <si>
@@ -261,9 +255,6 @@
     <t>cals2gains.com</t>
   </si>
   <si>
-    <t>TOTAL MENSUAL</t>
-  </si>
-  <si>
     <t>Plataforma</t>
   </si>
   <si>
@@ -406,6 +397,36 @@
   </si>
   <si>
     <t>Receipt-2466-5491-6579</t>
+  </si>
+  <si>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>ElevenLabs</t>
+  </si>
+  <si>
+    <t>Creator subscription (50% descuento 1er mes)</t>
+  </si>
+  <si>
+    <t>OY9NEJ2T-0001</t>
+  </si>
+  <si>
+    <t>15/04/2026</t>
+  </si>
+  <si>
+    <t>Receipt-2771-7868-1788 / Invoice-5RBPQUSE-0006</t>
+  </si>
+  <si>
+    <t>Creator (1er mes 50% off)</t>
+  </si>
+  <si>
+    <t>14/05/2026</t>
+  </si>
+  <si>
+    <t>Activa (enrollment 14/04/2026)</t>
+  </si>
+  <si>
+    <t>14/04/2027</t>
   </si>
 </sst>
 </file>
@@ -1291,7 +1312,7 @@
   <sheetPr>
     <tabColor rgb="FF1B2A4A"/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -1438,10 +1459,10 @@
         <v>46121</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>19</v>
@@ -1456,13 +1477,13 @@
         <v>20</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J5" s="19" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -1470,10 +1491,10 @@
         <v>46122</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>19</v>
@@ -1491,10 +1512,10 @@
         <v>14</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -1502,10 +1523,10 @@
         <v>46125</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D7" s="19" t="s">
         <v>19</v>
@@ -1520,24 +1541,24 @@
         <v>20</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J7" s="19" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="22" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D8" s="19" t="s">
         <v>19</v>
@@ -1555,19 +1576,79 @@
         <v>14</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="J8" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="D9" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E9" s="7">
-        <f>SUM(E2:E8)</f>
-        <v>1097.08</v>
+        <v>12.25</v>
+      </c>
+      <c r="F9">
+        <v>13.31</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>122</v>
+      </c>
+      <c r="B10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10">
+        <v>170</v>
+      </c>
+      <c r="F10">
+        <v>170</v>
+      </c>
+      <c r="G10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E11">
+        <v>1279.33</v>
       </c>
     </row>
   </sheetData>
@@ -1589,7 +1670,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>19</v>
@@ -1601,21 +1682,21 @@
         <v>26</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="9">
         <v>1057.0899999999999</v>
@@ -1642,7 +1723,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="10">
         <v>0</v>
@@ -1669,7 +1750,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="10">
         <v>0</v>
@@ -1696,7 +1777,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" s="10">
         <v>0</v>
@@ -1723,7 +1804,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="10">
         <v>0</v>
@@ -1750,7 +1831,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" s="10">
         <v>0</v>
@@ -1777,7 +1858,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" s="10">
         <v>0</v>
@@ -1804,7 +1885,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="10">
         <v>0</v>
@@ -1831,7 +1912,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" s="10">
         <v>0</v>
@@ -1858,7 +1939,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" s="12">
         <f>SUM(B2:B10)</f>
@@ -1894,7 +1975,7 @@
   <sheetPr>
     <tabColor rgb="FF548235"/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1905,36 +1986,36 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>52</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>53</v>
       </c>
       <c r="C2" s="9">
         <v>9.99</v>
@@ -1950,7 +2031,7 @@
         <v>46148</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>22</v>
@@ -1958,10 +2039,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>56</v>
       </c>
       <c r="C3" s="9">
         <v>16.989999999999998</v>
@@ -1977,7 +2058,7 @@
         <v>46154</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>22</v>
@@ -1985,10 +2066,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C4" s="9">
         <v>170</v>
@@ -2003,18 +2084,18 @@
         <v>46151</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>60</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>61</v>
       </c>
       <c r="C5" s="9">
         <v>20</v>
@@ -2026,18 +2107,18 @@
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>64</v>
       </c>
       <c r="C6" s="9">
         <v>6</v>
@@ -2049,18 +2130,18 @@
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>58</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>65</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>66</v>
       </c>
       <c r="C7" s="10">
         <f>D7/12</f>
@@ -2069,14 +2150,14 @@
       <c r="D7" s="9">
         <v>99</v>
       </c>
-      <c r="E7" s="13">
-        <v>46122</v>
-      </c>
-      <c r="F7" s="13">
-        <v>46487</v>
+      <c r="E7" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>127</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>67</v>
+        <v>126</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>22</v>
@@ -2084,10 +2165,10 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C8" s="9">
         <v>0</v>
@@ -2098,7 +2179,7 @@
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>15</v>
@@ -2106,33 +2187,54 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
       <c r="B10" s="6" t="s">
-        <v>72</v>
+        <v>124</v>
       </c>
       <c r="C10" s="7">
-        <f>SUM(C2:C9)</f>
-        <v>231.23</v>
+        <v>24.49</v>
       </c>
       <c r="D10" s="7">
-        <f>SUM(D2:D9)</f>
-        <v>2774.76</v>
+        <v>293.88</v>
+      </c>
+      <c r="E10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" t="s">
+        <v>125</v>
+      </c>
+      <c r="G10" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C11">
+        <v>255.72</v>
+      </c>
+      <c r="D11">
+        <v>3068.64</v>
       </c>
     </row>
   </sheetData>
@@ -2156,33 +2258,33 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -2217,27 +2319,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="24" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="25"/>
       <c r="C2" s="25"/>
@@ -2271,36 +2373,36 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -2314,7 +2416,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
@@ -2328,7 +2430,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
@@ -2342,7 +2444,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B5" s="10">
         <v>16.989999999999998</v>
@@ -2358,7 +2460,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B6" s="12">
         <v>0</v>
@@ -2386,7 +2488,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="14" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -2448,7 +2550,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="10">
         <v>0</v>
@@ -2464,7 +2566,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="10">
         <v>0</v>
@@ -2480,7 +2582,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14" s="10">
         <v>0</v>
@@ -2496,7 +2598,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B15" s="12">
         <v>502.08</v>
@@ -2524,7 +2626,7 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B17" s="12">
         <v>-502.08</v>
@@ -2540,7 +2642,7 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2554,7 +2656,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B19" s="10">
         <v>502.08</v>
@@ -2586,27 +2688,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="8"/>
@@ -2622,7 +2724,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="8"/>
@@ -2638,7 +2740,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="10"/>
       <c r="C4" s="8"/>
@@ -2654,7 +2756,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="8"/>
@@ -2670,7 +2772,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="8"/>
@@ -2686,7 +2788,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="8"/>
@@ -2702,7 +2804,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="8"/>
@@ -2718,7 +2820,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="8"/>
@@ -2734,7 +2836,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="8"/>
@@ -2766,7 +2868,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="20" x14ac:dyDescent="0.4">
       <c r="A1" s="28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
@@ -2778,19 +2880,19 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="29" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B3" s="25"/>
       <c r="C3" s="29" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D3" s="25"/>
       <c r="E3" s="29" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F3" s="25"/>
       <c r="G3" s="29" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="H3" s="25"/>
     </row>
@@ -2819,7 +2921,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -2851,7 +2953,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="18">
         <v>0</v>
@@ -2859,7 +2961,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="18">
         <v>0</v>
@@ -2867,7 +2969,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B12" s="18">
         <v>0</v>

</xml_diff>